<commit_message>
Update Naver Webtoon Series mapping
</commit_message>
<xml_diff>
--- a/data/adult_login_required_webtoons_v2.xlsx
+++ b/data/adult_login_required_webtoons_v2.xlsx
@@ -634,7 +634,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:38</t>
+          <t>2026-10-19 12:41:46</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:39</t>
+          <t>2026-10-19 12:41:46</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -926,26 +926,26 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>망플루언서</t>
+          <t>우리들의 속사정</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=850526&amp;tab=mon</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=855893&amp;tab=mon</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>850526</t>
+          <t>855893</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:39</t>
+          <t>2026-10-19 12:41:47</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -973,48 +973,204 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>우리들의 속사정</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>우리들의 속사정 (총 6화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>총 6화/미완결</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=14834100</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>14834100</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>우리들의 속사정 (총 6화/미완결)
+평점
+10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료
+모든 게 잘 맞지만 딱 하나! 속궁합이 맞지 않는다면?완벽한 궁합을 위해 고군분투하는 사회 초년생들의 웃픈 속사정 로맨스!</t>
+        </is>
+      </c>
+      <c r="Y4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mon</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>월</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>39</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>망플루언서</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=850526&amp;tab=mon</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>850526</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:47</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>mon</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>mon</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>망플루언서</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>망플루언서 (총 12화/미완결)</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>총 12화/미완결</t>
         </is>
       </c>
-      <c r="R4" t="n">
+      <c r="R5" t="n">
         <v>12</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>평점 10.0 | 망순 망순 | 2026.06.14. | 총12화/미완결 | 6화 무료</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>평점 10.0 | 망순 망순 | 2026.06.14. | 총12화/미완결 | 6화 무료</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14140191</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>14140191</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>망플루언서 (총 12화/미완결)
 평점
@@ -1022,155 +1178,155 @@
 대중의 관심을 먹고 사는 빛나는 직업 '인플루언서!'보여지는 모습과 달리 그들의 숨겨진 추악한 비밀들을 폭로하는 유명 렉카 너튜브 채널 '셀럽 쓰레기통'그 채널을 운영하는 두 여자, 선미와 주원의 이야기."거짓으로 돈을 ..</t>
         </is>
       </c>
-      <c r="Y4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA4" t="n">
+      <c r="Y5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA5" t="n">
         <v>105</v>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
+      <c r="AJ5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>월</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>57</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C6" t="n">
+        <v>59</v>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>피폐물을 힐링물로 만드는 방법</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=826381&amp;tab=mon</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>826381</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:40</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:47</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>피폐물을 힐링물로 만드는 방법</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>피폐물을 힐링물로 만드는 방법 (총 84화/미완결)</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>총 84화/미완결</t>
         </is>
       </c>
-      <c r="R5" t="n">
+      <c r="R6" t="n">
         <v>84</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>평점 9.9 | 류호, 황도톨 양담 | 2026.06.14. | 총84화/미완결 | 78화 무료</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>평점 9.9 | 류호, 황도톨 양담 | 2026.06.14. | 총84화/미완결 | 78화 무료</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=11152272</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>11152272</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>피폐물을 힐링물로 만드는 방법 (총 84화/미완결)
 평점
@@ -1178,161 +1334,161 @@
 [살아생전 즐겨보던 소설에 환생했다.] 너무 진부하다구요? 아닐 걸요!왜냐면 그 소설이... 19금 피폐물이거든요...! ̗̀(ꀬ⏖ꀬ∴)예쁘고 상냥한 여주인공의 동생으로 환생했지만, 언니의 새드엔딩을 지켜볼 수 없었던 레나티..</t>
         </is>
       </c>
-      <c r="Y5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA5" t="n">
+      <c r="Y6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="n">
         <v>105</v>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
-      <c r="AE5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF5" t="inlineStr">
+      <c r="AE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="inlineStr">
         <is>
           <t>216.7만</t>
         </is>
       </c>
-      <c r="AG5" t="n">
+      <c r="AG6" t="n">
         <v>2167000</v>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
+      <c r="AJ6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>월</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>61</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="C7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>페일 블루 아이즈</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=849898&amp;tab=mon</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>849898</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:40</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:47</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>페일 블루 아이즈</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>페일 블루 아이즈 (총 13화/미완결)</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>총 13화/미완결</t>
         </is>
       </c>
-      <c r="R6" t="n">
+      <c r="R7" t="n">
         <v>13</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>평점 9.9 | LICO, 피숙혜 당도삼십 | 2026.06.14. | 총13화/미완결 | 9화 무료</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>평점 9.9 | LICO, 피숙혜 당도삼십 | 2026.06.14. | 총13화/미완결 | 9화 무료</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14051143</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>14051143</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>페일 블루 아이즈 (총 13화/미완결)
 평점
@@ -1340,155 +1496,155 @@
 주은은 자신을 늘 외롭게 만드는 가족을 떠나 홀연히 영국으로 향한다. 그곳에서 만난 창백한 푸른눈의 남자, 에덴. 조악한 문신으로 온몸을 뒤덮은, 쓰레기 같은 펑크를 노래하는, 주변의 모든 여자를 열병에 들끓게 만드는, 하..</t>
         </is>
       </c>
-      <c r="Y6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA6" t="n">
+      <c r="Y7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA7" t="n">
         <v>105</v>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
+      <c r="AE7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK6" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
+      <c r="AJ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>월</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>88</v>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C8" t="n">
+        <v>87</v>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>누가 죄인인가</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=846782&amp;tab=mon</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>846782</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:41</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:48</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>mon</t>
         </is>
       </c>
-      <c r="N7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>누가 죄인인가</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>누가 죄인인가 (총 41화/미완결)</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>총 41화/미완결</t>
         </is>
       </c>
-      <c r="R7" t="n">
+      <c r="R8" t="n">
         <v>41</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>평점 10.0 | 이승우 이승우 | 2026.10.04. | 총41화/미완결 | 34화 무료</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>평점 10.0 | 이승우 이승우 | 2026.10.04. | 총41화/미완결 | 34화 무료</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=13634954</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>13634954</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>누가 죄인인가 (총 41화/미완결)
 평점
@@ -1496,162 +1652,6 @@
 "나의 아버지는 악마로 만들어졌다."연쇄살인마 '허욱열'의 딸로서 30년간 지옥 같은 삶을 살아온 일류 청부업자 '허예주' 오늘날 허욱열의 무고가 밝혀지게 되지만 이들은 여전히 지옥 속에 살고 있고 예주는자신과 같이 지옥 ..</t>
         </is>
       </c>
-      <c r="Y7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>mon</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>월</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>121</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>우리들의 속사정</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=855893&amp;tab=mon</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>855893</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:41</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>mon</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>mon</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>우리들의 속사정</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>우리들의 속사정 (총 6화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>총 6화/미완결</t>
-        </is>
-      </c>
-      <c r="R8" t="n">
-        <v>6</v>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=14834100</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>14834100</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>우리들의 속사정 (총 6화/미완결)
-평점
-10.0 | 강문송 아와와 | 2026.10.11. | 총6화/미완결 | 1화 무료
-모든 게 잘 맞지만 딱 하나! 속궁합이 맞지 않는다면?완벽한 궁합을 위해 고군분투하는 사회 초년생들의 웃픈 속사정 로맨스!</t>
-        </is>
-      </c>
       <c r="Y8" t="b">
         <v>0</v>
       </c>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>searched_series</t>
+          <t>reused_existing_product_no</t>
         </is>
       </c>
       <c r="AJ8" t="b">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:41</t>
+          <t>2026-10-19 12:41:49</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:49</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:49</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:50</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:50</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:50</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:42</t>
+          <t>2026-10-19 12:41:50</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2793,7 +2793,7 @@
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:43</t>
+          <t>2026-10-19 12:41:51</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:44</t>
+          <t>2026-10-19 12:41:52</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:44</t>
+          <t>2026-10-19 12:41:52</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:45</t>
+          <t>2026-10-19 12:41:52</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:45</t>
+          <t>2026-10-19 12:41:54</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:46</t>
+          <t>2026-10-19 12:41:54</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3764,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:46</t>
+          <t>2026-10-19 12:41:55</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:47</t>
+          <t>2026-10-19 12:41:55</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:48</t>
+          <t>2026-10-19 12:41:56</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:48</t>
+          <t>2026-10-19 12:41:56</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -4368,26 +4368,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>당신에게 얽힌 채</t>
+          <t>순결을 그대에게</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=849879&amp;tab=thu</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=821589&amp;tab=thu</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>849879</t>
+          <t>821589</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:48</t>
+          <t>2026-10-19 12:41:56</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -4415,48 +4415,204 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
+          <t>순결을 그대에게</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>순결을 그대에게 (총 29화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>총 29화/미완결</t>
+        </is>
+      </c>
+      <c r="R26" t="n">
+        <v>29</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=10749793</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>10749793</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>순결을 그대에게 (총 29화/미완결)
+평점
+10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료
+원치 않는 결혼을 피하기 위해 소꿉친구인 딘에게 순결을 잃으려는 세라.하지만 딘의 모습이 어딘가 서툴다.“너 혹시 처음이야?”주인과 하인. 신분 차이를 넘나드는 첫사랑 로맨스.</t>
+        </is>
+      </c>
+      <c r="Y26" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ26" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>목</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>75</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>당신에게 얽힌 채</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=849879&amp;tab=thu</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>849879</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:56</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>thu</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>당신에게 얽힌 채</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t>당신에게 얽힌 채 (총 10화/미완결)</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>총 10화/미완결</t>
         </is>
       </c>
-      <c r="R26" t="n">
+      <c r="R27" t="n">
         <v>10</v>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S27" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>평점 10.0 | Nicole Knight, 유다 danah789 | 2026.06.17. | 총10화/미완결 | 5화 무료</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14041685</t>
         </is>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="W27" t="inlineStr">
         <is>
           <t>14041685</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>당신에게 얽힌 채 (총 10화/미완결)
 평점
@@ -4464,162 +4620,6 @@
 상속자가 아닌 복종하는 존재로 길러진 에이바 모레티. 뉴욕에서 가장 강력한 마피아 가문의 막내딸인 그녀는 ‘집안의 사고뭉치’라는 오명을 벗고 자신의 자리를 찾기 위해 분투한다.그러던 어느 날 밤, 낯선 남자와 보낸 뜨..</t>
         </is>
       </c>
-      <c r="Y26" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z26" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI26" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ26" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK26" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>목</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>96</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>순결을 그대에게</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=821589&amp;tab=thu</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>821589</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:49</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="b">
-        <v>1</v>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>thu</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>순결을 그대에게</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>순결을 그대에게 (총 29화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>총 29화/미완결</t>
-        </is>
-      </c>
-      <c r="R27" t="n">
-        <v>29</v>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=10749793</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>10749793</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>순결을 그대에게 (총 29화/미완결)
-평점
-10.0 | 지공 지공 | 2024.07.31. | 총29화/미완결 | 전화 무료
-원치 않는 결혼을 피하기 위해 소꿉친구인 딘에게 순결을 잃으려는 세라.하지만 딘의 모습이 어딘가 서툴다.“너 혹시 처음이야?”주인과 하인. 신분 차이를 넘나드는 첫사랑 로맨스.</t>
-        </is>
-      </c>
       <c r="Y27" t="b">
         <v>0</v>
       </c>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>searched_series</t>
+          <t>reused_existing_product_no</t>
         </is>
       </c>
       <c r="AJ27" t="b">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:49</t>
+          <t>2026-10-19 12:41:57</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="AK28" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:49</t>
+          <t>2026-10-19 12:41:57</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:49</t>
+          <t>2026-10-19 12:41:57</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:49</t>
+          <t>2026-10-19 12:41:57</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="AK31" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:50</t>
+          <t>2026-10-19 12:41:58</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5466,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:50</t>
+          <t>2026-10-19 12:41:58</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5628,7 +5628,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:51</t>
+          <t>2026-10-19 12:41:59</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -5790,26 +5790,26 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>사탄의 순애</t>
+          <t>죽여주는 캐스팅</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=845378&amp;tab=fri</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=843866&amp;tab=fri</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>845378</t>
+          <t>843866</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:51</t>
+          <t>2026-10-19 12:41:59</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -5837,48 +5837,204 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
+          <t>죽여주는 캐스팅 [독점]</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>죽여주는 캐스팅 [독점] (총 42화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>총 42화/미완결</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>42</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>평점 9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>평점 9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=13253015</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>13253015</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>죽여주는 캐스팅 [독점] (총 42화/미완결)
+평점
+9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료
+영화감상 동호회에서 만난 혜수와 강호.성공한 배우를 꿈꾸는 강호는 오디션과 술자리에 몰두하며 혜수에게 기대어 살아간다.그런 강호를 이해하고자 혜수는 연기 수업을 시작하고 점차 자신의 길을 걷기 시작한다.하지만 강..</t>
+        </is>
+      </c>
+      <c r="Y35" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fri</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>금</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>79</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>사탄의 순애</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=845378&amp;tab=fri</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>845378</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:41:59</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>fri</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>fri</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
           <t>사탄의 순애 [독점]</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>사탄의 순애 [독점] (총 35화/미완결)</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>총 35화/미완결</t>
         </is>
       </c>
-      <c r="R35" t="n">
+      <c r="R36" t="n">
         <v>35</v>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>평점 9.8 | 용현 카모모 | 2026.06.18. | 총35화/미완결 | 28화 무료</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>평점 9.8 | 용현 카모모 | 2026.06.18. | 총35화/미완결 | 28화 무료</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr">
+      <c r="V36" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=13451638</t>
         </is>
       </c>
-      <c r="W35" t="inlineStr">
+      <c r="W36" t="inlineStr">
         <is>
           <t>13451638</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>사탄의 순애 [독점] (총 35화/미완결)
 평점
@@ -5886,162 +6042,6 @@
 초식동물계 대표주자 호구남 백은우 VS 육식동물계 대표주자 차도녀 범호연.정반대의 두 사람은 어쩌다 사귀게 됐을까?“백은우. 나한테 취업해라. 내 애인인 척 딱 1년. 그럼 10억이야.”업계에서 악마로 소문난 아티스트 레..</t>
         </is>
       </c>
-      <c r="Y35" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z35" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA35" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB35" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC35" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD35" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF35" t="inlineStr"/>
-      <c r="AG35" t="inlineStr"/>
-      <c r="AH35" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI35" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ35" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK35" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>fri</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>금</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>74</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>죽여주는 캐스팅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=843866&amp;tab=fri</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>843866</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:51</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="b">
-        <v>1</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>fri</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>fri</t>
-        </is>
-      </c>
-      <c r="N36" t="n">
-        <v>1</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>죽여주는 캐스팅 [독점]</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>죽여주는 캐스팅 [독점] (총 42화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>총 42화/미완결</t>
-        </is>
-      </c>
-      <c r="R36" t="n">
-        <v>42</v>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>평점 9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>평점 9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=13253015</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>13253015</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>죽여주는 캐스팅 [독점] (총 42화/미완결)
-평점
-9.6 | 영춘 하보 | 2026.06.18. | 총42화/미완결 | 36화 무료
-영화감상 동호회에서 만난 혜수와 강호.성공한 배우를 꿈꾸는 강호는 오디션과 술자리에 몰두하며 혜수에게 기대어 살아간다.그런 강호를 이해하고자 혜수는 연기 수업을 시작하고 점차 자신의 길을 걷기 시작한다.하지만 강..</t>
-        </is>
-      </c>
       <c r="Y36" t="b">
         <v>0</v>
       </c>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6121,7 +6121,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:52</t>
+          <t>2026-10-19 12:42:00</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:52</t>
+          <t>2026-10-19 12:42:00</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:52</t>
+          <t>2026-10-19 12:42:00</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -6553,7 +6553,7 @@
       </c>
       <c r="AK39" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6569,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:53</t>
+          <t>2026-10-19 12:42:00</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="AK40" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:53</t>
+          <t>2026-10-19 12:42:01</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="AK41" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -6880,26 +6880,26 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>데스루프</t>
+          <t>메이드</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=852086&amp;tab=sat</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=854905&amp;tab=sat</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>852086</t>
+          <t>854905</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:54</t>
+          <t>2026-10-19 12:42:01</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -6927,48 +6927,210 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
+          <t>마이 페어 메이드</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>마이 페어 메이드 (총 85화/완결)</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>총 85화/완결</t>
+        </is>
+      </c>
+      <c r="R42" t="n">
+        <v>85</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>완결</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>평점 9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>평점 9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=8033729</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>8033729</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>마이 페어 메이드 (총 85화/완결)
+평점
+9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료
+특기가 청소인 귀여운 메이드 샌디, 까칠한 바람둥이 도련님 킬리언의 약혼녀가 되다!어느 번개 치던 날 사교계 최고 미녀인 알렉산드라에게 빙의 된 샌디.평소 침 흘리며 바라보던 공작가 도련님 킬리언의 약혼녀가 되어 있다..</t>
+        </is>
+      </c>
+      <c r="Y42" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z42" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>first_non_compilation_numeric_download</t>
+        </is>
+      </c>
+      <c r="AE42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>93만</t>
+        </is>
+      </c>
+      <c r="AG42" t="n">
+        <v>930000</v>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ42" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>sat</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>토</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>67</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>데스루프</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=852086&amp;tab=sat</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>852086</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:42:01</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="b">
+        <v>1</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>sat</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>sat</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>1</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>데스루프</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
         <is>
           <t>데스루프 (총 6화/미완결)</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>총 6화/미완결</t>
         </is>
       </c>
-      <c r="R42" t="n">
+      <c r="R43" t="n">
         <v>6</v>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>미완결</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>평점 8.3 | 은삼 은삼 | 2026.06.26. | 총6화/미완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>평점 8.3 | 은삼 은삼 | 2026.06.26. | 총6화/미완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14366954</t>
         </is>
       </c>
-      <c r="W42" t="inlineStr">
+      <c r="W43" t="inlineStr">
         <is>
           <t>14366954</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>데스루프 (총 6화/미완결)
 평점
@@ -6976,162 +7138,6 @@
 정신을 차려 보니 지하 창고에 갇힌 주인공 홍연화.연화는 자신을 가둔 남성에게 여러 번 끔찍한 죽음을 맞이하지만, 계속해서 시간이 반복된다.겨우 그곳을 빠져나오지만 그녀 앞에 마주한 것은 끔찍하게 생긴 괴물.과연 그녀..</t>
         </is>
       </c>
-      <c r="Y42" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z42" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA42" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB42" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC42" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD42" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE42" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF42" t="inlineStr"/>
-      <c r="AG42" t="inlineStr"/>
-      <c r="AH42" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI42" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ42" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK42" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>sat</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>토</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>80</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>메이드</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=854905&amp;tab=sat</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>854905</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:54</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="b">
-        <v>1</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>sat</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>sat</t>
-        </is>
-      </c>
-      <c r="N43" t="n">
-        <v>1</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>마이 페어 메이드</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>마이 페어 메이드 (총 85화/완결)</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>총 85화/완결</t>
-        </is>
-      </c>
-      <c r="R43" t="n">
-        <v>85</v>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>완결</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>평점 9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>평점 9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료</t>
-        </is>
-      </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=8033729</t>
-        </is>
-      </c>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>8033729</t>
-        </is>
-      </c>
-      <c r="X43" t="inlineStr">
-        <is>
-          <t>마이 페어 메이드 (총 85화/완결)
-평점
-9.8 | 솔체/DIAN 샌도 | 2023.09.29. | 총85화/완결 | 3화 무료
-특기가 청소인 귀여운 메이드 샌디, 까칠한 바람둥이 도련님 킬리언의 약혼녀가 되다!어느 번개 치던 날 사교계 최고 미녀인 알렉산드라에게 빙의 된 샌디.평소 침 흘리며 바라보던 공작가 도련님 킬리언의 약혼녀가 되어 있다..</t>
-        </is>
-      </c>
       <c r="Y43" t="b">
         <v>0</v>
       </c>
@@ -7148,33 +7154,27 @@
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>matched</t>
+          <t>review_needed</t>
         </is>
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>first_non_compilation_numeric_download</t>
+          <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
       <c r="AE43" t="n">
         <v>1</v>
       </c>
-      <c r="AF43" t="inlineStr">
-        <is>
-          <t>93만</t>
-        </is>
-      </c>
-      <c r="AG43" t="n">
-        <v>930000</v>
-      </c>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="AI43" t="inlineStr">
         <is>
-          <t>searched_series</t>
+          <t>reused_existing_product_no</t>
         </is>
       </c>
       <c r="AJ43" t="b">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="AK43" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:55</t>
+          <t>2026-10-19 12:42:03</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:56</t>
+          <t>2026-10-19 12:42:03</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -7494,7 +7494,7 @@
       </c>
       <c r="AK45" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:56</t>
+          <t>2026-10-19 12:42:03</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="AK46" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -7684,7 +7684,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:56</t>
+          <t>2026-10-19 12:42:03</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="AK47" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -7821,26 +7821,26 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>나의 비발디</t>
+          <t>적귀</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=854344&amp;tab=sun</t>
+          <t>https://comic.naver.com/webtoon/list?titleId=855665&amp;tab=sun</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>854344</t>
+          <t>855665</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:56</t>
+          <t>2026-10-19 12:42:03</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -7864,16 +7864,16 @@
         </is>
       </c>
       <c r="N48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>나의 비발디</t>
+          <t>적귀</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>나의 비발디 (총 6화/미완결)</t>
+          <t>적귀 (총 6화/미완결)</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -7891,25 +7891,181 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
+          <t>평점 10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>평점 10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=14812060</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>14812060</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>적귀 (총 6화/미완결)
+평점
+10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료
+폭력과 욕망이 들끓던 1980년대. 임광천과 조도원, 두 남자가 뒷세계에 도전장을 내민다. 그들은 목표는 전국의 주먹을 꺾고 누구도 올라서지 못했던 정점. “전국제패” 〈부활남〉, 〈한림체육관〉의 최강자 임광천, 그의 전..</t>
+        </is>
+      </c>
+      <c r="Y48" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z48" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_2</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF48" t="inlineStr"/>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ48" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>47</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>나의 비발디</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=854344&amp;tab=sun</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>854344</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:42:04</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="b">
+        <v>1</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>1</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>나의 비발디</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>나의 비발디 (총 6화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>총 6화/미완결</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>6</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
           <t>평점 10.0 | 배청이 틸다123 | 2026.09.05. | 총6화/미완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>평점 10.0 | 배청이 틸다123 | 2026.09.05. | 총6화/미완결 | 1화 무료</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
+      <c r="V49" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=14580181</t>
         </is>
       </c>
-      <c r="W48" t="inlineStr">
+      <c r="W49" t="inlineStr">
         <is>
           <t>14580181</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>나의 비발디 (총 6화/미완결)
 평점
@@ -7917,155 +8073,311 @@
 "갖고 싶어... 가르쳐줘, 네 재능."천재의 재능을 훔쳐 정상에 오른 피아니스트 윤설아.그리고 버려진 천재, 우지환.홀로 신곡을 발표한 설아는 추락하고,복수를 결심한 지환은 다시 그녀의 앞에 나타난다.이번엔, 내가 널 가질 차..</t>
         </is>
       </c>
-      <c r="Y48" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z48" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA48" t="n">
+      <c r="Y49" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z49" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA49" t="n">
         <v>105</v>
       </c>
-      <c r="AB48" t="inlineStr">
+      <c r="AB49" t="inlineStr">
         <is>
           <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
         </is>
       </c>
-      <c r="AC48" t="inlineStr">
+      <c r="AC49" t="inlineStr">
         <is>
           <t>review_needed</t>
         </is>
       </c>
-      <c r="AD48" t="inlineStr">
+      <c r="AD49" t="inlineStr">
         <is>
           <t>non_compilation_but_download_not_ok</t>
         </is>
       </c>
-      <c r="AE48" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF48" t="inlineStr"/>
-      <c r="AG48" t="inlineStr"/>
-      <c r="AH48" t="inlineStr">
+      <c r="AE49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr">
         <is>
           <t>not_found</t>
         </is>
       </c>
-      <c r="AI48" t="inlineStr">
+      <c r="AI49" t="inlineStr">
         <is>
           <t>reused_existing_product_no</t>
         </is>
       </c>
-      <c r="AJ48" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK48" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
+      <c r="AJ49" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C49" t="n">
-        <v>42</v>
-      </c>
-      <c r="D49" t="inlineStr">
+      <c r="C50" t="n">
+        <v>48</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>지옥심판</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://comic.naver.com/webtoon/list?titleId=854096&amp;tab=sun</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>854096</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:42:04</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="b">
+        <v>1</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>login_or_adult_required</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>1</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>지옥심판</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>지옥심판 (총 7화/미완결)</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>총 7화/미완결</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
+        <v>7</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>미완결</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>평점 9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>평점 9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>https://series.naver.com/comic/detail.series?productNo=14622042</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>14622042</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>지옥심판 (총 7화/미완결)
+평점
+9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료
+죄를 지은 인간은 언젠가 벌을 받게 되어있다. 이승이 아닌 저승에서라도.죄인을 심판하고 지옥으로 인도하는 저승사자 이현의 이야기.</t>
+        </is>
+      </c>
+      <c r="Y50" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z50" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>105</v>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>review_needed</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>non_compilation_but_download_not_ok</t>
+        </is>
+      </c>
+      <c r="AE50" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>reused_existing_product_no</t>
+        </is>
+      </c>
+      <c r="AJ50" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>2026-10-19 13:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>51</v>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>인터뷰</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>https://comic.naver.com/webtoon/list?titleId=854396&amp;tab=sun</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>854396</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:56</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="b">
-        <v>1</v>
-      </c>
-      <c r="J49" t="inlineStr">
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:42:04</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="b">
+        <v>1</v>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>login_or_adult_required</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M51" t="inlineStr">
         <is>
           <t>sun</t>
         </is>
       </c>
-      <c r="N49" t="n">
-        <v>1</v>
-      </c>
-      <c r="O49" t="inlineStr">
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
+      <c r="O51" t="inlineStr">
         <is>
           <t>살인자와의 인터뷰 [개정판][컬러연재]</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>살인자와의 인터뷰 [개정판][컬러연재] (총 53화/완결)</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="Q51" t="inlineStr">
         <is>
           <t>총 53화/완결</t>
         </is>
       </c>
-      <c r="R49" t="n">
+      <c r="R51" t="n">
         <v>53</v>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="S51" t="inlineStr">
         <is>
           <t>완결</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="T51" t="inlineStr">
         <is>
           <t>평점 9.9 | KJK KJK | 2019.04.10. | 총53화/완결 | 4화 무료</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>평점 9.9 | KJK KJK | 2019.04.10. | 총53화/완결 | 4화 무료</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr">
+      <c r="V51" t="inlineStr">
         <is>
           <t>https://series.naver.com/comic/detail.series?productNo=3181357</t>
         </is>
       </c>
-      <c r="W49" t="inlineStr">
+      <c r="W51" t="inlineStr">
         <is>
           <t>3181357</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>살인자와의 인터뷰 [개정판][컬러연재] (총 53화/완결)
 평점
@@ -8073,324 +8385,6 @@
 특종보다는 흥미를 느끼는 취재거리만 찾는 도윤에게 구 남친이 연락해 귀가 솔깃한 제안을 한다.바로 자신의 심리치료 환자인 연쇄 살인범과의 인터뷰를 진행하는 것.자신의 은밀한 사생활(?!)을 유지하고 싶었던 도윤은 이 ..</t>
         </is>
       </c>
-      <c r="Y49" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z49" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA49" t="n">
-        <v>105</v>
-      </c>
-      <c r="AB49" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_1</t>
-        </is>
-      </c>
-      <c r="AC49" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="AD49" t="inlineStr">
-        <is>
-          <t>first_non_compilation_numeric_download</t>
-        </is>
-      </c>
-      <c r="AE49" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF49" t="inlineStr">
-        <is>
-          <t>30.1만</t>
-        </is>
-      </c>
-      <c r="AG49" t="n">
-        <v>301000</v>
-      </c>
-      <c r="AH49" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AI49" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ49" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK49" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>44</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>적귀</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=855665&amp;tab=sun</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>855665</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:56</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="b">
-        <v>1</v>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="N50" t="n">
-        <v>2</v>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>적귀</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>적귀 (총 6화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>총 6화/미완결</t>
-        </is>
-      </c>
-      <c r="R50" t="n">
-        <v>6</v>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T50" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>평점 10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=14812060</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>14812060</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>적귀 (총 6화/미완결)
-평점
-10.0 | 혜성 이석재 | 2026.10.03. | 총6화/미완결 | 1화 무료
-폭력과 욕망이 들끓던 1980년대. 임광천과 조도원, 두 남자가 뒷세계에 도전장을 내민다. 그들은 목표는 전국의 주먹을 꺾고 누구도 올라서지 못했던 정점. “전국제패” 〈부활남〉, 〈한림체육관〉의 최강자 임광천, 그의 전..</t>
-        </is>
-      </c>
-      <c r="Y50" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z50" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA50" t="n">
-        <v>100</v>
-      </c>
-      <c r="AB50" t="inlineStr">
-        <is>
-          <t>title_contains,bonus_total_episode_info,bonus_rank_2</t>
-        </is>
-      </c>
-      <c r="AC50" t="inlineStr">
-        <is>
-          <t>review_needed</t>
-        </is>
-      </c>
-      <c r="AD50" t="inlineStr">
-        <is>
-          <t>non_compilation_but_download_not_ok</t>
-        </is>
-      </c>
-      <c r="AE50" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF50" t="inlineStr"/>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr">
-        <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="AI50" t="inlineStr">
-        <is>
-          <t>reused_existing_product_no</t>
-        </is>
-      </c>
-      <c r="AJ50" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK50" t="inlineStr">
-        <is>
-          <t>2026-10-12 14:31:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>47</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>지옥심판</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>https://comic.naver.com/webtoon/list?titleId=854096&amp;tab=sun</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>854096</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>2026-10-12 13:49:56</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="b">
-        <v>1</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>login_or_adult_required</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>sun</t>
-        </is>
-      </c>
-      <c r="N51" t="n">
-        <v>1</v>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>지옥심판</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>지옥심판 (총 7화/미완결)</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>총 7화/미완결</t>
-        </is>
-      </c>
-      <c r="R51" t="n">
-        <v>7</v>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>미완결</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>평점 9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>평점 9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>https://series.naver.com/comic/detail.series?productNo=14622042</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>14622042</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>지옥심판 (총 7화/미완결)
-평점
-9.6 | 가강 주혁 | 2026.08.22. | 총7화/미완결 | 2화 무료
-죄를 지은 인간은 언젠가 벌을 받게 되어있다. 이승이 아닌 저승에서라도.죄인을 심판하고 지옥으로 인도하는 저승사자 이현의 이야기.</t>
-        </is>
-      </c>
       <c r="Y51" t="b">
         <v>0</v>
       </c>
@@ -8407,22 +8401,28 @@
       </c>
       <c r="AC51" t="inlineStr">
         <is>
-          <t>review_needed</t>
+          <t>matched</t>
         </is>
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>non_compilation_but_download_not_ok</t>
+          <t>first_non_compilation_numeric_download</t>
         </is>
       </c>
       <c r="AE51" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF51" t="inlineStr"/>
-      <c r="AG51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>30.1만</t>
+        </is>
+      </c>
+      <c r="AG51" t="n">
+        <v>301000</v>
+      </c>
       <c r="AH51" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AI51" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="AK51" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -8451,7 +8451,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:57</t>
+          <t>2026-10-19 12:42:04</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -8597,7 +8597,7 @@
       </c>
       <c r="AK52" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:57</t>
+          <t>2026-10-19 12:42:04</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="AK53" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -8769,7 +8769,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:58</t>
+          <t>2026-10-19 12:42:05</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="AK54" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>
@@ -8925,7 +8925,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-10-12 13:49:58</t>
+          <t>2026-10-19 12:42:05</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="AK55" t="inlineStr">
         <is>
-          <t>2026-10-12 14:31:25</t>
+          <t>2026-10-19 13:25:54</t>
         </is>
       </c>
     </row>

</xml_diff>